<commit_message>
Evaluation done again. Place : Institute.
</commit_message>
<xml_diff>
--- a/Interrater_Agreement_1.xlsx
+++ b/Interrater_Agreement_1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\docs\Projects\PythonProject\UStoria\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\docs\Projects\UStoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C34D902-9581-4F04-896F-783B4E5E7D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6350" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Per_Criterion" sheetId="1" r:id="rId1"/>
@@ -137,7 +138,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -493,17 +494,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -520,7 +521,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -537,7 +538,7 @@
         <v>-3.899606946677681E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -554,7 +555,7 @@
         <v>1.423082491701266E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -571,7 +572,7 @@
         <v>2.675436698365341E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -585,7 +586,7 @@
         <v>-5.5099608969446656E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -602,7 +603,7 @@
         <v>3.339441968002399E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -619,7 +620,7 @@
         <v>-5.0240119199149724E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -636,7 +637,7 @@
         <v>9.8190000066269434E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -656,15 +657,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
@@ -681,7 +685,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -698,7 +702,7 @@
         <v>2.2187406200805389E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -715,7 +719,7 @@
         <v>-2.086074826485262E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -732,7 +736,7 @@
         <v>-2.7340311498258441E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -749,7 +753,7 @@
         <v>1.3638098287077629E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -766,7 +770,7 @@
         <v>-2.9276598489498258E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -789,17 +793,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -816,7 +820,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>

</xml_diff>